<commit_message>
Update dependencies and add XLSM regression tests
- migrate to Rust 2024 and umya-spreadsheet 3.0
- track Cargo.lock and move trycmd to dev-dependencies
- report workbook read failures as CLI errors
- add macro-enabled workbook and formatting regression coverage

Known issue: Excel-compatible date/time formatting currently fails
due to umya-spreadsheet number format handling.
</commit_message>
<xml_diff>
--- a/tests/test.xlsx
+++ b/tests/test.xlsx
@@ -4,15 +4,16 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="test_sheet" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
+    <sheet name="シート4" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
   <si>
     <t>test1</t>
   </si>
@@ -131,6 +132,83 @@
   </si>
   <si>
     <t>end3</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>テスト</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>テスト</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+4</t>
+    </r>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>時刻</t>
+    <rPh sb="0" eb="2">
+      <t>ジコク</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>日付</t>
+    <rPh sb="0" eb="2">
+      <t>ヒヅケ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>aaa</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>bbb</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>ccc</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>-</t>
     <phoneticPr fontId="3"/>
   </si>
 </sst>
@@ -138,7 +216,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4">
+  <numFmts count="4">
+    <numFmt numFmtId="177" formatCode="yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;;@"/>
+    <numFmt numFmtId="178" formatCode="m&quot;月&quot;d&quot;日&quot;;@"/>
+    <numFmt numFmtId="181" formatCode="0.0_);[Red]\(0.0\)"/>
+    <numFmt numFmtId="182" formatCode="0.0_ "/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Noto Sans CJK JP"/>
@@ -160,6 +244,20 @@
     </font>
     <font>
       <sz val="6"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Noto Sans CJK JP"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="ＭＳ Ｐゴシック"/>
       <family val="3"/>
       <charset val="128"/>
@@ -206,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -218,6 +316,28 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="32" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -311,13 +431,13 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>180975</xdr:colOff>
+          <xdr:colOff>184150</xdr:colOff>
           <xdr:row>0</xdr:row>
           <xdr:rowOff>57150</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>638175</xdr:colOff>
+          <xdr:colOff>641350</xdr:colOff>
           <xdr:row>2</xdr:row>
           <xdr:rowOff>19050</xdr:rowOff>
         </xdr:to>
@@ -342,7 +462,7 @@
             </a:prstGeom>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="36576" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="ctr" rtl="0">
@@ -670,9 +790,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="12"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="25.5">
+    <row r="1" spans="1:4" ht="26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -686,7 +806,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="12.75">
+    <row r="2" spans="1:4" ht="12.5">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -720,13 +840,13 @@
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
                     <xdr:col>4</xdr:col>
-                    <xdr:colOff>180975</xdr:colOff>
+                    <xdr:colOff>184150</xdr:colOff>
                     <xdr:row>0</xdr:row>
                     <xdr:rowOff>57150</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>638175</xdr:colOff>
+                    <xdr:colOff>641350</xdr:colOff>
                     <xdr:row>2</xdr:row>
                     <xdr:rowOff>19050</xdr:rowOff>
                   </to>
@@ -744,9 +864,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B3:J9"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="12"/>
   <sheetData>
-    <row r="3" spans="2:10" ht="25.5">
+    <row r="3" spans="2:10" ht="26">
       <c r="G3" s="1" t="s">
         <v>6</v>
       </c>
@@ -760,7 +880,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:10" ht="12.75">
+    <row r="4" spans="2:10" ht="12.5">
       <c r="G4" s="3" t="s">
         <v>8</v>
       </c>
@@ -774,7 +894,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="12.75">
+    <row r="5" spans="2:10" ht="12.5">
       <c r="G5" s="3" t="s">
         <v>12</v>
       </c>
@@ -788,7 +908,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:10" ht="25.5">
+    <row r="7" spans="2:10" ht="26">
       <c r="B7" s="1" t="s">
         <v>0</v>
       </c>
@@ -805,24 +925,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:10" ht="12.75">
+    <row r="8" spans="2:10" ht="12.5">
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="11">
         <v>3</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="11">
         <v>4</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:10" ht="12.75">
+    <row r="9" spans="2:10" ht="12.5">
       <c r="B9" s="3" t="s">
         <v>16</v>
       </c>
@@ -855,7 +975,7 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="12"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="25.5">
+    <row r="1" spans="1:5" ht="26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -884,7 +1004,7 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="12"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="25.5">
+    <row r="1" spans="1:5" ht="26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -912,8 +1032,8 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="4"/>
-      <c r="B3" s="4">
-        <v>2</v>
+      <c r="B3" s="12">
+        <v>2.2999999999999998</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -1076,5 +1196,79 @@
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="12"/>
+  <cols>
+    <col min="3" max="3" width="16.59765625" customWidth="1"/>
+    <col min="4" max="4" width="14.796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="26">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="12.5">
+      <c r="A2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="6">
+        <v>0.6875</v>
+      </c>
+      <c r="C2" s="7">
+        <v>46156</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="12.5">
+      <c r="A3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C3" s="9">
+        <v>46156</v>
+      </c>
+      <c r="D3" s="8">
+        <f>B3-B2</f>
+        <v>6.25E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="12.5">
+      <c r="A4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="C4" s="10">
+        <v>46156</v>
+      </c>
+      <c r="D4" s="8">
+        <f>B4-B3</f>
+        <v>8.333333333333337E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>